<commit_message>
Various changes involving websocket connections.
Made timer which stops all tank operations when no command has been received for 1s and message is now sent to server when sensor is hit.
</commit_message>
<xml_diff>
--- a/Hardware Calcs.xlsx
+++ b/Hardware Calcs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vicke\Documents\2026-ECSE-Design-Comp\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\quila\Local_Projects\ECSE\ECSE_Design_Competition_2\2026-ECSE-Design-Comp\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{755C7818-A529-4539-B030-E96C1B68CB04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -223,7 +223,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -244,12 +244,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -615,18 +609,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B2:I15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="24.5703125" customWidth="1"/>
-    <col min="3" max="3" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="20.7109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.54296875" customWidth="1"/>
+    <col min="3" max="3" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.26953125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="20.7265625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:9" ht="21" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:9" ht="21" x14ac:dyDescent="0.5">
       <c r="B2" s="4" t="s">
         <v>0</v>
       </c>
@@ -640,7 +634,7 @@
       </c>
       <c r="I2" s="4"/>
     </row>
-    <row r="4" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B4" t="s">
         <v>6</v>
       </c>
@@ -661,7 +655,7 @@
         <v>38000</v>
       </c>
     </row>
-    <row r="5" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:9" x14ac:dyDescent="0.35">
       <c r="E5" t="s">
         <v>5</v>
       </c>
@@ -669,7 +663,7 @@
         <v>0.3</v>
       </c>
     </row>
-    <row r="6" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:9" x14ac:dyDescent="0.35">
       <c r="E6" t="s">
         <v>11</v>
       </c>
@@ -677,7 +671,7 @@
         <v>0.6</v>
       </c>
     </row>
-    <row r="7" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B7" t="s">
         <v>3</v>
       </c>
@@ -692,7 +686,7 @@
         <v>0.93</v>
       </c>
     </row>
-    <row r="8" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B8" t="s">
         <v>14</v>
       </c>
@@ -708,7 +702,7 @@
         <v>9.9999999999999995E-7</v>
       </c>
     </row>
-    <row r="12" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C12" t="s">
         <v>8</v>
       </c>
@@ -716,7 +710,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B13" t="s">
         <v>10</v>
       </c>
@@ -729,7 +723,7 @@
         <v>4.4444444444444447E-5</v>
       </c>
     </row>
-    <row r="14" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B14" t="s">
         <v>13</v>
       </c>
@@ -742,7 +736,7 @@
         <v>2.52E-6</v>
       </c>
     </row>
-    <row r="15" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B15" t="s">
         <v>12</v>
       </c>
@@ -769,18 +763,18 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F4BF82C-C0F2-4F6F-8968-BBCA72124B8C}">
   <dimension ref="B2:I15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="24.5703125" customWidth="1"/>
-    <col min="3" max="3" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="20.7109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.54296875" customWidth="1"/>
+    <col min="3" max="3" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.26953125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="20.7265625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:9" ht="21" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:9" ht="21" x14ac:dyDescent="0.5">
       <c r="B2" s="4" t="s">
         <v>0</v>
       </c>
@@ -794,7 +788,7 @@
       </c>
       <c r="I2" s="4"/>
     </row>
-    <row r="4" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B4" t="s">
         <v>6</v>
       </c>
@@ -815,7 +809,7 @@
         <v>38000</v>
       </c>
     </row>
-    <row r="5" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:9" x14ac:dyDescent="0.35">
       <c r="E5" t="s">
         <v>5</v>
       </c>
@@ -829,7 +823,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="6" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:9" x14ac:dyDescent="0.35">
       <c r="E6" t="s">
         <v>11</v>
       </c>
@@ -837,7 +831,7 @@
         <v>0.6</v>
       </c>
     </row>
-    <row r="7" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B7" t="s">
         <v>3</v>
       </c>
@@ -852,7 +846,7 @@
         <v>0.93</v>
       </c>
     </row>
-    <row r="8" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B8" t="s">
         <v>14</v>
       </c>
@@ -868,7 +862,7 @@
         <v>9.9999999999999995E-7</v>
       </c>
     </row>
-    <row r="12" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C12" t="s">
         <v>8</v>
       </c>
@@ -876,7 +870,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B13" t="s">
         <v>10</v>
       </c>
@@ -889,7 +883,7 @@
         <v>4.4444444444444447E-5</v>
       </c>
     </row>
-    <row r="14" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B14" t="s">
         <v>13</v>
       </c>
@@ -902,7 +896,7 @@
         <v>2.52E-6</v>
       </c>
     </row>
-    <row r="15" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B15" t="s">
         <v>12</v>
       </c>

</xml_diff>